<commit_message>
Add team tournament support #1
</commit_message>
<xml_diff>
--- a/docs/technical-appendices/chess-results/Tie-Breaks.xlsx
+++ b/docs/technical-appendices/chess-results/Tie-Breaks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20415"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\Daten\SwissManager\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\Daten\SwissManager\NeueTieBreak_Rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D78B56A5-F76D-45E4-B49D-E99047B5E2B9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F8FF8D-DEDD-4BE5-AE2C-871E5E04233E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="26850" windowHeight="9135" xr2:uid="{7A6EA089-5FA8-4040-BFAD-5CA2839738CF}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="224">
   <si>
     <t>points (game-points)</t>
   </si>
@@ -543,9 +543,6 @@
     <t>S</t>
   </si>
   <si>
-    <t>S …. Only available in Swiss-Chess</t>
-  </si>
-  <si>
     <t>B …  For Playerperformance list/Board list in Team-Tournaments</t>
   </si>
   <si>
@@ -606,9 +603,6 @@
     <t>discarded weakest results</t>
   </si>
   <si>
-    <t>1200,0,0</t>
-  </si>
-  <si>
     <t>- or P</t>
   </si>
   <si>
@@ -667,6 +661,42 @@
   </si>
   <si>
     <t>MP,P</t>
+  </si>
+  <si>
+    <t>Type 0..WIN, 1…WON, 2..BWG, 3..BPG</t>
+  </si>
+  <si>
+    <t>Fore Buchholz</t>
+  </si>
+  <si>
+    <t>Kashdan</t>
+  </si>
+  <si>
+    <t>Kas</t>
+  </si>
+  <si>
+    <t>S …. Only available in Swiss-Chess or other Programs</t>
+  </si>
+  <si>
+    <t>Parameter 6</t>
+  </si>
+  <si>
+    <t>Parameter 7</t>
+  </si>
+  <si>
+    <t>Valid from 1.2.2026</t>
+  </si>
+  <si>
+    <t>Valid from 1.2.2026: 1 or 0</t>
+  </si>
+  <si>
+    <t>Take in account unplayed games</t>
+  </si>
+  <si>
+    <t>Take in account unplayed games: 1 or 0</t>
+  </si>
+  <si>
+    <t>1200,0,0,0</t>
   </si>
 </sst>
 </file>
@@ -1054,7 +1084,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E1D5251-9B61-4D3E-B085-3401CC1CA7A6}">
-  <dimension ref="A1:U101"/>
+  <dimension ref="A1:V101"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" bestFit="1" customWidth="1"/>
@@ -1065,7 +1095,10 @@
     <col min="9" max="9" width="13.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.140625" customWidth="1"/>
+    <col min="15" max="15" width="18" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.42578125" style="6"/>
+    <col min="21" max="21" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="99.75" x14ac:dyDescent="0.25">
@@ -1094,24 +1127,28 @@
         <v>160</v>
       </c>
       <c r="I1" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="M1" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
+      <c r="N1" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>218</v>
+      </c>
       <c r="P1" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -2782,6 +2819,15 @@
       <c r="H69" s="4" t="s">
         <v>154</v>
       </c>
+      <c r="I69" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="J69" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q69" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70">
@@ -2973,24 +3019,24 @@
         <v>169</v>
       </c>
       <c r="I77" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="J77" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="J77" s="4" t="s">
+      <c r="K77" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="K77" s="4" t="s">
+      <c r="L77" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="L77" s="4" t="s">
+      <c r="M77" s="4" t="s">
         <v>182</v>
-      </c>
-      <c r="M77" s="4" t="s">
-        <v>183</v>
       </c>
       <c r="N77" s="4"/>
       <c r="O77" s="4"/>
       <c r="P77" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.25">
@@ -3019,13 +3065,13 @@
         <v>169</v>
       </c>
       <c r="I78" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>154</v>
       </c>
       <c r="Q78" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.25">
@@ -3054,7 +3100,7 @@
         <v>169</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.25">
@@ -3083,10 +3129,10 @@
         <v>154</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.25">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="81" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -3112,19 +3158,25 @@
         <v>154</v>
       </c>
       <c r="I81" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="J81" t="s">
+        <v>206</v>
+      </c>
+      <c r="K81" t="s">
         <v>191</v>
       </c>
-      <c r="J81" t="s">
-        <v>208</v>
-      </c>
-      <c r="K81" t="s">
-        <v>192</v>
+      <c r="L81" s="4" t="s">
+        <v>221</v>
       </c>
       <c r="P81" s="6" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="82" spans="1:21" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+      <c r="T81" s="6" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="82" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -3150,16 +3202,16 @@
         <v>154</v>
       </c>
       <c r="I82" s="7" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="Q82" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="83" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -3188,28 +3240,28 @@
         <v>161</v>
       </c>
       <c r="J83" t="s">
+        <v>206</v>
+      </c>
+      <c r="K83" t="s">
+        <v>191</v>
+      </c>
+      <c r="L83" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="M83" t="s">
+        <v>207</v>
+      </c>
+      <c r="P83" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q83" t="s">
+        <v>194</v>
+      </c>
+      <c r="U83" t="s">
         <v>208</v>
       </c>
-      <c r="K83" t="s">
-        <v>192</v>
-      </c>
-      <c r="L83" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="M83" t="s">
-        <v>209</v>
-      </c>
-      <c r="P83" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="Q83" t="s">
-        <v>196</v>
-      </c>
-      <c r="U83" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="84" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="84" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -3235,19 +3287,19 @@
         <v>169</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J84" s="7" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="P84" s="6" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="Q84" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="85" spans="1:21" x14ac:dyDescent="0.25">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="85" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -3276,32 +3328,37 @@
         <v>161</v>
       </c>
       <c r="J85" t="s">
+        <v>206</v>
+      </c>
+      <c r="K85" t="s">
+        <v>191</v>
+      </c>
+      <c r="L85" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="M85" t="s">
+        <v>213</v>
+      </c>
+      <c r="N85" t="s">
+        <v>207</v>
+      </c>
+      <c r="O85" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="P85" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="Q85" t="s">
+        <v>198</v>
+      </c>
+      <c r="U85" t="s">
         <v>208</v>
       </c>
-      <c r="K85" t="s">
-        <v>192</v>
-      </c>
-      <c r="L85" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="M85" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="N85" t="s">
-        <v>209</v>
-      </c>
-      <c r="O85" s="7"/>
-      <c r="P85" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="Q85" t="s">
-        <v>200</v>
-      </c>
-      <c r="U85" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V85" s="8" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="86" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -3330,19 +3387,19 @@
         <v>0</v>
       </c>
       <c r="J86" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K86" t="s">
+        <v>191</v>
+      </c>
+      <c r="L86" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="L86" s="7" t="s">
-        <v>194</v>
-      </c>
       <c r="P86" s="6" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="87" spans="1:21" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="87" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -3371,16 +3428,16 @@
         <v>161</v>
       </c>
       <c r="J87" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="P87" s="8" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="Q87" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="88" spans="1:21" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="88" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -3409,16 +3466,16 @@
         <v>161</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P88" s="8" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="Q88" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="89" spans="1:21" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="89" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -3447,16 +3504,16 @@
         <v>161</v>
       </c>
       <c r="J89" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P89" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="Q89" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="90" spans="1:21" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="90" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -3482,13 +3539,13 @@
         <v>169</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="91" spans="1:21" x14ac:dyDescent="0.25">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="91" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -3514,18 +3571,18 @@
         <v>169</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="92" spans="1:21" x14ac:dyDescent="0.25">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="92" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C92" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>156</v>
@@ -3543,18 +3600,44 @@
         <v>169</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J92" s="7" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="94" spans="1:21" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="93" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>214</v>
+      </c>
+      <c r="C93" t="s">
+        <v>215</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G93" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="H93" s="4" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="94" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C94" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="95" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>167</v>
       </c>
@@ -3562,7 +3645,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="96" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
         <v>162</v>
       </c>
@@ -3584,15 +3667,16 @@
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
-        <v>172</v>
+        <v>216</v>
       </c>
     </row>
     <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>